<commit_message>
Customer page - excel
</commit_message>
<xml_diff>
--- a/src/test/resources/dataTest/dataProjectCuoiKhoa.xlsx
+++ b/src/test/resources/dataTest/dataProjectCuoiKhoa.xlsx
@@ -8,13 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\anhTester\Project_Cuoi_Khoa\src\test\resources\dataTest\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5F7565E5-F42B-4F54-B75B-42624D601925}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{743F988A-5D3F-4291-A995-88B5FBCFBAB2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336" xr2:uid="{D4AABB89-EE12-468A-B216-C59207BCAFCF}"/>
+    <workbookView xWindow="3144" yWindow="3360" windowWidth="17280" windowHeight="8880" activeTab="1" xr2:uid="{D4AABB89-EE12-468A-B216-C59207BCAFCF}"/>
   </bookViews>
   <sheets>
-    <sheet name="Customers" sheetId="1" r:id="rId1"/>
-    <sheet name="Projects" sheetId="2" r:id="rId2"/>
+    <sheet name="Login" sheetId="3" r:id="rId1"/>
+    <sheet name="Customer" sheetId="1" r:id="rId2"/>
+    <sheet name="Project" sheetId="2" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -40,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="39">
   <si>
     <t>Project_Name</t>
   </si>
@@ -69,9 +70,6 @@
     <t>Company</t>
   </si>
   <si>
-    <t>VAT_Number</t>
-  </si>
-  <si>
     <t>Phone</t>
   </si>
   <si>
@@ -112,13 +110,61 @@
   </si>
   <si>
     <t>VietNam</t>
+  </si>
+  <si>
+    <t>10</t>
+  </si>
+  <si>
+    <t>7000</t>
+  </si>
+  <si>
+    <t>TCs</t>
+  </si>
+  <si>
+    <t>Email</t>
+  </si>
+  <si>
+    <t>Password</t>
+  </si>
+  <si>
+    <t>loginSuccess</t>
+  </si>
+  <si>
+    <t>admin@example.com</t>
+  </si>
+  <si>
+    <t>123456</t>
+  </si>
+  <si>
+    <t>admin123@example.com</t>
+  </si>
+  <si>
+    <t>2222222</t>
+  </si>
+  <si>
+    <t>loginFailWithEmailInvalid</t>
+  </si>
+  <si>
+    <t>loginFailWithPassInvalid</t>
+  </si>
+  <si>
+    <t>VAT</t>
+  </si>
+  <si>
+    <t>Status</t>
+  </si>
+  <si>
+    <t>Passed</t>
+  </si>
+  <si>
+    <t>Công ty Ween</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -126,13 +172,28 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="8"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="3" tint="0.89999084444715716"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="none"/>
     </fill>
   </fills>
   <borders count="1">
@@ -147,8 +208,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -482,77 +548,144 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B1129EC2-D029-48F9-827C-BCE01AB8E176}">
-  <dimension ref="A1:J2"/>
-  <sheetFormatPr defaultColWidth="16.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D93C7CD2-8E73-43DE-94E6-3A28F5CAF450}">
+  <dimension ref="A1:C4"/>
+  <sheetFormatPr defaultColWidth="21.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>8</v>
+        <v>25</v>
       </c>
       <c r="B1" t="s">
-        <v>9</v>
+        <v>26</v>
       </c>
       <c r="C1" t="s">
-        <v>10</v>
-      </c>
-      <c r="D1" t="s">
-        <v>11</v>
-      </c>
-      <c r="E1" t="s">
-        <v>12</v>
-      </c>
-      <c r="F1" t="s">
-        <v>13</v>
-      </c>
-      <c r="G1" t="s">
-        <v>14</v>
-      </c>
-      <c r="H1" t="s">
-        <v>15</v>
-      </c>
-      <c r="I1" t="s">
-        <v>16</v>
-      </c>
-      <c r="J1" t="s">
-        <v>17</v>
+        <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="B2">
-        <v>10</v>
-      </c>
-      <c r="C2" t="s">
-        <v>18</v>
-      </c>
-      <c r="D2" t="s">
-        <v>19</v>
-      </c>
-      <c r="E2" t="s">
-        <v>20</v>
-      </c>
-      <c r="F2" t="s">
-        <v>21</v>
-      </c>
-      <c r="G2" t="s">
-        <v>21</v>
-      </c>
-      <c r="H2" t="s">
-        <v>22</v>
-      </c>
-      <c r="I2">
-        <v>7000</v>
-      </c>
-      <c r="J2" t="s">
-        <v>23</v>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>28</v>
+      </c>
+      <c r="B2" t="s">
+        <v>29</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>33</v>
+      </c>
+      <c r="B3" t="s">
+        <v>31</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>34</v>
+      </c>
+      <c r="B4" t="s">
+        <v>29</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>32</v>
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B1129EC2-D029-48F9-827C-BCE01AB8E176}">
+  <dimension ref="A1:K3"/>
+  <sheetFormatPr defaultColWidth="16.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData>
+    <row r="1" spans="1:11" s="2" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="I1" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="J1" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="K1" s="2" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>38</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="C2" t="s">
+        <v>17</v>
+      </c>
+      <c r="D2" t="s">
+        <v>18</v>
+      </c>
+      <c r="E2" t="s">
+        <v>19</v>
+      </c>
+      <c r="F2" t="s">
+        <v>20</v>
+      </c>
+      <c r="G2" t="s">
+        <v>20</v>
+      </c>
+      <c r="H2" t="s">
+        <v>21</v>
+      </c>
+      <c r="I2" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="J2" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="K3" s="3" t="s">
+        <v>37</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{84FC15DE-0E0A-485E-AD31-E7992A0D7BD7}">
   <dimension ref="A1:H1"/>
   <sheetFormatPr defaultColWidth="16.5546875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>

</xml_diff>

<commit_message>
xml parallel full project
</commit_message>
<xml_diff>
--- a/src/test/resources/dataTest/dataProjectCuoiKhoa.xlsx
+++ b/src/test/resources/dataTest/dataProjectCuoiKhoa.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\anhTester\Project_Cuoi_Khoa\src\test\resources\dataTest\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{70230AE2-7041-4CA6-B0ED-D659B755BDF0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{29DDE3D3-9DFB-46A7-A48E-DB707E572B44}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{D4AABB89-EE12-468A-B216-C59207BCAFCF}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{D4AABB89-EE12-468A-B216-C59207BCAFCF}"/>
   </bookViews>
   <sheets>
     <sheet name="Login" sheetId="3" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="145" uniqueCount="110">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="155" uniqueCount="111">
   <si>
     <t>Project_Name</t>
   </si>
@@ -372,6 +372,9 @@
   </si>
   <si>
     <t>AssigneesProject ManagerAdmin Anh TesterAdmin Example</t>
+  </si>
+  <si>
+    <t>11</t>
   </si>
 </sst>
 </file>
@@ -857,7 +860,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B1129EC2-D029-48F9-827C-BCE01AB8E176}">
-  <dimension ref="A1:N3"/>
+  <dimension ref="A1:N4"/>
   <sheetFormatPr defaultColWidth="21.5546875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:14" s="2" customFormat="1" x14ac:dyDescent="0.3">
@@ -980,6 +983,38 @@
         <v>62</v>
       </c>
       <c r="L3" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="4" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="B4" s="1" t="s">
+        <v>110</v>
+      </c>
+      <c r="C4" t="s">
+        <v>57</v>
+      </c>
+      <c r="D4" t="s">
+        <v>58</v>
+      </c>
+      <c r="E4" t="s">
+        <v>17</v>
+      </c>
+      <c r="F4" t="s">
+        <v>47</v>
+      </c>
+      <c r="G4" t="s">
+        <v>48</v>
+      </c>
+      <c r="H4" t="s">
+        <v>61</v>
+      </c>
+      <c r="I4" t="s">
+        <v>61</v>
+      </c>
+      <c r="K4" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="L4" t="s">
         <v>63</v>
       </c>
     </row>

</xml_diff>